<commit_message>
Add word "forfalden" to Pipi.xlsx
</commit_message>
<xml_diff>
--- a/sets/Pipi.xlsx
+++ b/sets/Pipi.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -517,9 +517,95 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>3a9f37ff-49c4-42ab-84b8-0c0439a141ec</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-07-27</v>
+      </c>
+      <c r="C2" t="str">
+        <v>forfalden</v>
+      </c>
+      <c r="D2" t="str">
+        <v>forfalden</v>
+      </c>
+      <c r="E2" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>-t, forfaldne</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[fʌˈfalˀən]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014469_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>i dårlig stand (pga. manglende vedligeholdelse)</v>
+      </c>
+      <c r="K2" t="str">
+        <v>overdue</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v>| Biblioteket Sønderborg</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=8e81801b-12c1-47fd-8369-ee111821c1a4</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://biblioteket.sonderborg.dk/reader?orderid=8e81801b-12c1-47fd-8369-ee111821c1a4#:~:text=forfalden</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -528,28 +614,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -631,8 +717,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add phrase "føre til" to Pipi.xlsx
</commit_message>
<xml_diff>
--- a/sets/Pipi.xlsx
+++ b/sets/Pipi.xlsx
@@ -401,34 +401,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -612,30 +612,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -706,9 +706,77 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>9e5fe3de-8765-4535-a6e9-9296ce7afde1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-07-27</v>
+      </c>
+      <c r="C2" t="str">
+        <v>føre til</v>
+      </c>
+      <c r="D2" t="str">
+        <v>føre=lead · til=to</v>
+      </c>
+      <c r="E2" t="str">
+        <v>lead to</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Kan føre til skader på boligen: Specialist efterlyser skærpede krav til solceller</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://ing.dk/#:~:text=f%C3%B8re%20til</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Afgørende" to Pipi.xlsx
</commit_message>
<xml_diff>
--- a/sets/Pipi.xlsx
+++ b/sets/Pipi.xlsx
@@ -399,36 +399,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -603,9 +603,95 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>333bacb2-93b9-4490-9baa-4693ea103c92</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-07-27</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Afgørende</v>
+      </c>
+      <c r="D3" t="str">
+        <v>afgørende</v>
+      </c>
+      <c r="E3" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>-, -</v>
+      </c>
+      <c r="H3" t="str">
+        <v>[-ˌgɶˀʌnə]</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://static.ordnet.dk/mp3/11000/11000442_1.mp3</v>
+      </c>
+      <c r="J3" t="str">
+        <v>se afgøre</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Conclusive</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Afgørende beskyttelse af forpint hav har stået stille i to år: »Det er dybt kritisabelt«</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://ing.dk/#:~:text=Afg%C3%B8rende</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -614,28 +700,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Phone: delete 1 in Pipi.xlsx
</commit_message>
<xml_diff>
--- a/sets/Pipi.xlsx
+++ b/sets/Pipi.xlsx
@@ -88,106 +88,46 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -195,66 +135,27 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -263,136 +164,29 @@
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -401,34 +195,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB3"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -698,30 +492,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V1"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -792,77 +586,9 @@
         <v>Lapses_EN</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>9e5fe3de-8765-4535-a6e9-9296ce7afde1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2026-07-27</v>
-      </c>
-      <c r="C2" t="str">
-        <v>føre til</v>
-      </c>
-      <c r="D2" t="str">
-        <v>føre=lead · til=to</v>
-      </c>
-      <c r="E2" t="str">
-        <v>lead to</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Kan føre til skader på boligen: Specialist efterlyser skærpede krav til solceller</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Ingeniøren - nyheder om teknologi og samfund</v>
-      </c>
-      <c r="H2" t="str">
-        <v>https://ing.dk/</v>
-      </c>
-      <c r="I2" t="str">
-        <v>https://ing.dk/#:~:text=f%C3%B8re%20til</v>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v>ok</v>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
-      <c r="U2" t="str">
-        <v/>
-      </c>
-      <c r="V2" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress 1, log 1 in Pipi.xlsx
</commit_message>
<xml_diff>
--- a/sets/Pipi.xlsx
+++ b/sets/Pipi.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Words" sheetId="1" r:id="rId1"/>
     <sheet name="Phrases" sheetId="2" r:id="rId2"/>
     <sheet name="Meta" sheetId="3" r:id="rId3"/>
+    <sheet name="ReviewLog" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -193,36 +194,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AH2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="11.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -310,6 +317,24 @@
       <c r="AB1" t="str">
         <v>Lapses_EN</v>
       </c>
+      <c r="AC1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>LastReview</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Stability_EN</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Difficulty_EN</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>LastReview_EN</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -367,19 +392,19 @@
         <v/>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>2026-07-30</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="U2" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X2" t="str">
         <v/>
@@ -395,18 +420,27 @@
       </c>
       <c r="AB2" t="str">
         <v/>
+      </c>
+      <c r="AC2" t="str">
+        <v>3.17</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>5.28</v>
+      </c>
+      <c r="AE2" t="str">
+        <v>2026-07-27</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:AB1"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="10.83203125"/>
     <col min="2" max="2" customWidth="1" width="11.83203125"/>
@@ -430,6 +464,12 @@
     <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
     <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
     <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="23" max="23" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="11.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,10 +539,28 @@
       <c r="V1" t="str">
         <v>Lapses_EN</v>
       </c>
+      <c r="W1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>LastReview</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Stability_EN</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Difficulty_EN</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>LastReview_EN</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -552,4 +610,77 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Dir</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Time</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Grade</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Elapsed</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Interval</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>3a9f37ff-49c4-42ab-84b8-0c0439a141ec</v>
+      </c>
+      <c r="B2" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-07-27T19:26:26.217Z</v>
+      </c>
+      <c r="D2" t="str">
+        <v>good</v>
+      </c>
+      <c r="E2" t="str">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v>3.17</v>
+      </c>
+      <c r="G2" t="str">
+        <v>5.28</v>
+      </c>
+      <c r="H2" t="str">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add word "dræber" to Pipi.xlsx
</commit_message>
<xml_diff>
--- a/sets/Pipi.xlsx
+++ b/sets/Pipi.xlsx
@@ -89,46 +89,106 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -136,27 +196,66 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -165,71 +264,178 @@
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH2"/>
+  <dimension ref="A1:AH3"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="30" max="30" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="31" max="31" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="32" max="32" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="33" max="33" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="34" max="34" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -431,9 +637,113 @@
         <v>2026-07-27</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>84012969-f875-4303-9258-bbe80b133427</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="C3" t="str">
+        <v>dræber</v>
+      </c>
+      <c r="D3" t="str">
+        <v>dræber</v>
+      </c>
+      <c r="E3" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F3" t="str">
+        <v>en</v>
+      </c>
+      <c r="G3" t="str">
+        <v>-en, -e, -ne</v>
+      </c>
+      <c r="H3" t="str">
+        <v>[ˈdʁεːbʌ]</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://static.ordnet.dk/mp3/11009/11009809_1.mp3</v>
+      </c>
+      <c r="J3" t="str">
+        <v>nogen eller noget der slår ihjel (på en voldsom måde) eller på anden måde forårsager andres død</v>
+      </c>
+      <c r="K3" t="str">
+        <v>kills</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Jeg dræber ingenting!</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Jeg dræber ingenting! | Videos &amp; Movies on Vimeo</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://vimeo.com/1206503404?fl=pl&amp;fe=ti</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://vimeo.com/1206503404?fl=pl&amp;fe=ti#:~:text=dr%C3%A6ber</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+      <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
+        <v/>
+      </c>
+      <c r="AG3" t="str">
+        <v/>
+      </c>
+      <c r="AH3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -464,12 +774,12 @@
     <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
     <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
     <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="23" max="23" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="11.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -616,14 +926,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="12.83203125"/>
+    <col min="2" max="2" customWidth="1" width="12.83203125"/>
+    <col min="3" max="3" customWidth="1" width="12.83203125"/>
+    <col min="4" max="4" customWidth="1" width="12.83203125"/>
+    <col min="5" max="5" customWidth="1" width="12.83203125"/>
+    <col min="6" max="6" customWidth="1" width="12.83203125"/>
+    <col min="7" max="7" customWidth="1" width="12.83203125"/>
+    <col min="8" max="8" customWidth="1" width="12.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "alvorligt" to Pipi.xlsx
</commit_message>
<xml_diff>
--- a/sets/Pipi.xlsx
+++ b/sets/Pipi.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH3"/>
+  <dimension ref="A1:AH4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -741,9 +741,113 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>4f0e9221-8202-4e2e-b8fd-fee33eef092a</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="C4" t="str">
+        <v>alvorligt</v>
+      </c>
+      <c r="D4" t="str">
+        <v>alvorlig</v>
+      </c>
+      <c r="E4" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H4" t="str">
+        <v>[alˈvɒˀli]</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001475_1.mp3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>bekymrende; kritisk; farlig</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Seriously</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Maria Reumert Gjerding (SF) gav blandt andet en »king of trawlfree zones«-trøje til Magnus Heunicke i gave under ministeroverddragelsen i juni. I dag tager hun kritikken alvorligt og havde gerne set, at man var længere: »Min linje er klar: Der skal tempo på.« Illustration: Keld Navntoft/Ritzau Scanpix.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Fiskere trawler løs i kommende forbudszoner, viser ny data: »Havbunden kan ikke klare mere« | Ingeniøren</v>
+      </c>
+      <c r="N4" t="str">
+        <v>https://ing.dk/artikel/fiskere-trawler-loes-i-kommende-forbudszoner-viser-ny-data-havbunden-kan-ikke-klare-mere</v>
+      </c>
+      <c r="O4" t="str">
+        <v>https://ing.dk/artikel/fiskere-trawler-loes-i-kommende-forbudszoner-viser-ny-data-havbunden-kan-ikke-klare-mere#:~:text=alvorligt</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4" t="str">
+        <v/>
+      </c>
+      <c r="AE4" t="str">
+        <v/>
+      </c>
+      <c r="AF4" t="str">
+        <v/>
+      </c>
+      <c r="AG4" t="str">
+        <v/>
+      </c>
+      <c r="AH4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>